<commit_message>
Fixed CIMLR cluster names
</commit_message>
<xml_diff>
--- a/Results/single_algorithm/CIMLR/CIMLR_TCGA_RNAseq-CNV-Methylation-miRNA-SNPs_eval_on_transNEO_clusterings.xlsx
+++ b/Results/single_algorithm/CIMLR/CIMLR_TCGA_RNAseq-CNV-Methylation-miRNA-SNPs_eval_on_transNEO_clusterings.xlsx
@@ -23,7 +23,7 @@
     <t xml:space="preserve">TCGA-AQ-A0Y5-01A</t>
   </si>
   <si>
-    <t xml:space="preserve">CIMLRCIMLR1</t>
+    <t xml:space="preserve">CIMLR1</t>
   </si>
   <si>
     <t xml:space="preserve">TCGA-EW-A2FW-01A</t>
@@ -32,7 +32,7 @@
     <t xml:space="preserve">TCGA-C8-A274-01A</t>
   </si>
   <si>
-    <t xml:space="preserve">CIMLRCIMLR2</t>
+    <t xml:space="preserve">CIMLR2</t>
   </si>
   <si>
     <t xml:space="preserve">TCGA-B6-A0IK-01A</t>

</xml_diff>